<commit_message>
first pass at calibration for Matlab
</commit_message>
<xml_diff>
--- a/calibration/CalibrationDatafile_prevax 3.xlsx
+++ b/calibration/CalibrationDatafile_prevax 3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliciakraay/Dropbox/RotavirusVE_PamelaAlicia/ProposedProjects/Bangladesh data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliciakraay/PycharmProjects/rotasim/calibration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2050DFB1-E180-ED43-8135-C139FBEC653B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB6432F-3563-4243-BCBF-4BF9CA8696C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5260" yWindow="4660" windowWidth="26040" windowHeight="14940" activeTab="3" xr2:uid="{C5260B54-9666-D54D-BEE2-B441C4FA991D}"/>
+    <workbookView xWindow="3720" yWindow="3940" windowWidth="26040" windowHeight="14940" activeTab="7" xr2:uid="{C5260B54-9666-D54D-BEE2-B441C4FA991D}"/>
   </bookViews>
   <sheets>
     <sheet name="Dhaka_ageincidence" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Matlab_ageincidence" sheetId="3" r:id="rId4"/>
     <sheet name="Matlab_yr_geno" sheetId="4" r:id="rId5"/>
     <sheet name="Matlab_geno_mean" sheetId="5" r:id="rId6"/>
+    <sheet name="Matlab_incidence" sheetId="7" r:id="rId7"/>
+    <sheet name="Matlab_agedistribution" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="20">
   <si>
     <t>Age</t>
   </si>
@@ -98,6 +100,9 @@
   </si>
   <si>
     <t>ref_prop</t>
+  </si>
+  <si>
+    <t>[0, 125)</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD5E573-6851-7F4E-9CA7-51B823735174}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -1138,12 +1143,12 @@
         <v>204</v>
       </c>
       <c r="D2">
-        <f>240000*0.025</f>
-        <v>6000</v>
+        <f>240000*0.026</f>
+        <v>6240</v>
       </c>
       <c r="E2">
         <f>(C2/(D2*8))*100000</f>
-        <v>425.00000000000006</v>
+        <v>408.65384615384619</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1157,12 +1162,12 @@
         <v>150</v>
       </c>
       <c r="D3">
-        <f>240000*0.025</f>
-        <v>6000</v>
+        <f>240000*0.026</f>
+        <v>6240</v>
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E5" si="0">(C3/(D3*8))*100000</f>
-        <v>312.5</v>
+        <v>300.48076923076923</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1176,12 +1181,12 @@
         <v>21</v>
       </c>
       <c r="D4">
-        <f>240000*0.075</f>
-        <v>18000</v>
+        <f>240000*0.079</f>
+        <v>18960</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>14.583333333333334</v>
+        <v>13.844936708860761</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1195,12 +1200,18 @@
         <v>16</v>
       </c>
       <c r="D5">
-        <f>240000*0.875</f>
-        <v>210000</v>
+        <f>240000*0.869</f>
+        <v>208560</v>
       </c>
       <c r="E5">
         <f t="shared" si="0"/>
-        <v>0.95238095238095233</v>
+        <v>0.95895665515918671</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C6">
+        <f>SUM(C2:C5)</f>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -1732,4 +1743,138 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E0D8AEC-1468-E447-859B-E557AB4C5AE4}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <f>SUM(Matlab_ageincidence!C2:C5)</f>
+        <v>391</v>
+      </c>
+      <c r="D2">
+        <f>SUM(Matlab_ageincidence!D2:D5)</f>
+        <v>240000</v>
+      </c>
+      <c r="E2">
+        <f>(C2/(D2*8))*100000</f>
+        <v>20.364583333333332</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31FDD37E-C803-FD40-8D37-8B0B8BEFDC6F}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>204</v>
+      </c>
+      <c r="D2">
+        <f>C2/SUM(C2:C5)</f>
+        <v>0.52173913043478259</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>150</v>
+      </c>
+      <c r="D3">
+        <f>C3/SUM(C2:C5)</f>
+        <v>0.38363171355498721</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4">
+        <v>21</v>
+      </c>
+      <c r="D4">
+        <f>C4/SUM(C2:C5)</f>
+        <v>5.3708439897698211E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <f>C5/SUM(C2:C5)</f>
+        <v>4.0920716112531973E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>